<commit_message>
refactor: align category examples across documentation, visualization, and excel analysis
- use one representative category per segment (high-value, skewed, basket, mid-range)
- update README and data notes for consistent examples
- adjust scatter plot labels for clarity
- update excel workbook to reflect selected categories
</commit_message>
<xml_diff>
--- a/order_value_analysis.xlsx
+++ b/order_value_analysis.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adam/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adam/DataGripProjects/olist-ecommerce-analysis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB8E28D8-3932-C84B-A7BD-FA160E2EA8A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C384F188-E7FC-AD43-8F24-7B72E1F79FF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38560" yWindow="680" windowWidth="37920" windowHeight="40920" xr2:uid="{712AB7B1-C989-984F-A437-7028F968EAFA}"/>
+    <workbookView xWindow="520" yWindow="680" windowWidth="37920" windowHeight="19540" activeTab="2" xr2:uid="{712AB7B1-C989-984F-A437-7028F968EAFA}"/>
   </bookViews>
   <sheets>
     <sheet name="item_count_analysis" sheetId="1" r:id="rId1"/>
@@ -1636,12 +1636,18 @@
           <c:dLbls>
             <c:dLbl>
               <c:idx val="0"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="1.4366718986411007E-2"/>
+                  <c:y val="-2.9976707205496965E-17"/>
+                </c:manualLayout>
+              </c:layout>
               <c:tx>
                 <c:rich>
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{A8547637-2450-F549-8292-98EB1010639B}" type="CELLRANGE">
+                    <a:fld id="{7F841884-7CE2-8443-805F-093857D2D994}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -1650,8 +1656,9 @@
                   </a:p>
                 </c:rich>
               </c:tx>
+              <c:dLblPos val="r"/>
               <c:showLegendKey val="0"/>
-              <c:showVal val="1"/>
+              <c:showVal val="0"/>
               <c:showCatName val="0"/>
               <c:showSerName val="0"/>
               <c:showPercent val="0"/>
@@ -1668,32 +1675,9 @@
             </c:dLbl>
             <c:dLbl>
               <c:idx val="1"/>
-              <c:tx>
-                <c:rich>
-                  <a:bodyPr/>
-                  <a:lstStyle/>
-                  <a:p>
-                    <a:fld id="{2FE41838-EF65-AD4E-A283-00921E8B0CB0}" type="CELLRANGE">
-                      <a:rPr lang="en-US"/>
-                      <a:pPr/>
-                      <a:t>[CELLRANGE]</a:t>
-                    </a:fld>
-                    <a:endParaRPr lang="en-US"/>
-                  </a:p>
-                </c:rich>
-              </c:tx>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="0"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
+              <c:delete val="1"/>
               <c:extLst>
-                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                  <c15:dlblFieldTable/>
-                  <c15:xForSave val="1"/>
-                  <c15:showDataLabelsRange val="1"/>
-                </c:ext>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                   <c16:uniqueId val="{0000000D-6CF6-2543-89FD-1692317E3C47}"/>
                 </c:ext>
@@ -1711,12 +1695,18 @@
             </c:dLbl>
             <c:dLbl>
               <c:idx val="3"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="1.6162558859712382E-2"/>
+                  <c:y val="0"/>
+                </c:manualLayout>
+              </c:layout>
               <c:tx>
                 <c:rich>
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{6FB149B4-C1DE-5948-89C9-B15156B4C6E9}" type="CELLRANGE">
+                    <a:fld id="{426D681E-4AA1-8740-8C12-5F3AB28D6CB6}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -1725,6 +1715,7 @@
                   </a:p>
                 </c:rich>
               </c:tx>
+              <c:dLblPos val="r"/>
               <c:showLegendKey val="0"/>
               <c:showVal val="0"/>
               <c:showCatName val="0"/>
@@ -1734,7 +1725,6 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
-                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1744,32 +1734,9 @@
             </c:dLbl>
             <c:dLbl>
               <c:idx val="4"/>
-              <c:tx>
-                <c:rich>
-                  <a:bodyPr/>
-                  <a:lstStyle/>
-                  <a:p>
-                    <a:fld id="{0CA21BD2-510C-E543-90D4-77F120B2202B}" type="CELLRANGE">
-                      <a:rPr lang="en-US"/>
-                      <a:pPr/>
-                      <a:t>[CELLRANGE]</a:t>
-                    </a:fld>
-                    <a:endParaRPr lang="en-US"/>
-                  </a:p>
-                </c:rich>
-              </c:tx>
-              <c:showLegendKey val="0"/>
-              <c:showVal val="0"/>
-              <c:showCatName val="0"/>
-              <c:showSerName val="0"/>
-              <c:showPercent val="0"/>
-              <c:showBubbleSize val="0"/>
+              <c:delete val="1"/>
               <c:extLst>
-                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                  <c15:dlblFieldTable/>
-                  <c15:xForSave val="1"/>
-                  <c15:showDataLabelsRange val="1"/>
-                </c:ext>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                   <c16:uniqueId val="{00000010-6CF6-2543-89FD-1692317E3C47}"/>
                 </c:ext>
@@ -1787,12 +1754,28 @@
             </c:dLbl>
             <c:dLbl>
               <c:idx val="6"/>
+              <c:delete val="1"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000012-6CF6-2543-89FD-1692317E3C47}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="7"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="2.6937598099520604E-2"/>
+                  <c:y val="-4.2512912234912291E-2"/>
+                </c:manualLayout>
+              </c:layout>
               <c:tx>
                 <c:rich>
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{BB13094C-0857-7B4B-8C7A-C3AC6142B260}" type="CELLRANGE">
+                    <a:fld id="{20253A67-E322-BB4C-87D2-CBFE9B0025F0}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -1801,6 +1784,7 @@
                   </a:p>
                 </c:rich>
               </c:tx>
+              <c:dLblPos val="r"/>
               <c:showLegendKey val="0"/>
               <c:showVal val="0"/>
               <c:showCatName val="0"/>
@@ -1810,19 +1794,8 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                   <c15:dlblFieldTable/>
-                  <c15:xForSave val="1"/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
-                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                  <c16:uniqueId val="{00000012-6CF6-2543-89FD-1692317E3C47}"/>
-                </c:ext>
-              </c:extLst>
-            </c:dLbl>
-            <c:dLbl>
-              <c:idx val="7"/>
-              <c:delete val="1"/>
-              <c:extLst>
-                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                   <c16:uniqueId val="{00000013-6CF6-2543-89FD-1692317E3C47}"/>
                 </c:ext>
@@ -1860,15 +1833,27 @@
             </c:dLbl>
             <c:dLbl>
               <c:idx val="11"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="2.155007847961651E-2"/>
+                  <c:y val="0"/>
+                </c:manualLayout>
+              </c:layout>
               <c:tx>
                 <c:rich>
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
+                    <a:fld id="{C69A76CD-1558-2A4B-9140-8D572D3DDC8A}" type="CELLRANGE">
+                      <a:rPr lang="en-US"/>
+                      <a:pPr/>
+                      <a:t>[CELLRANGE]</a:t>
+                    </a:fld>
                     <a:endParaRPr lang="en-US"/>
                   </a:p>
                 </c:rich>
               </c:tx>
+              <c:dLblPos val="r"/>
               <c:showLegendKey val="0"/>
               <c:showVal val="0"/>
               <c:showCatName val="0"/>
@@ -1877,7 +1862,7 @@
               <c:showBubbleSize val="0"/>
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                  <c15:xForSave val="1"/>
+                  <c15:dlblFieldTable/>
                   <c15:showDataLabelsRange val="1"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
@@ -1914,6 +1899,7 @@
                 <a:endParaRPr lang="en-DE"/>
               </a:p>
             </c:txPr>
+            <c:dLblPos val="r"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="0"/>
             <c:showCatName val="0"/>
@@ -2036,9 +2022,9 @@
           <c:extLst>
             <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
               <c15:datalabelsRange>
-                <c15:f>category_analysis!$B$61:$B$71</c15:f>
+                <c15:f>category_analysis!$B$61:$B$72</c15:f>
                 <c15:dlblRangeCache>
-                  <c:ptCount val="11"/>
+                  <c:ptCount val="12"/>
                   <c:pt idx="0">
                     <c:v>pcs</c:v>
                   </c:pt>
@@ -2071,6 +2057,9 @@
                   </c:pt>
                   <c:pt idx="10">
                     <c:v>telefonia_fixa</c:v>
+                  </c:pt>
+                  <c:pt idx="11">
+                    <c:v>casa_conforto</c:v>
                   </c:pt>
                 </c15:dlblRangeCache>
               </c15:datalabelsRange>
@@ -4711,15 +4700,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>6679</xdr:colOff>
+      <xdr:colOff>6680</xdr:colOff>
       <xdr:row>73</xdr:row>
       <xdr:rowOff>13369</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>20053</xdr:colOff>
-      <xdr:row>90</xdr:row>
-      <xdr:rowOff>167106</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>6686</xdr:colOff>
+      <xdr:row>92</xdr:row>
+      <xdr:rowOff>86895</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>

</xml_diff>